<commit_message>
docs: add A3 to-do PDF and A4 phases-flowchart PDF
- mitsue_phases_funding_flowchart.pdf: 2-page A4 portrait, rendered from the
  Mermaid markdown with Liberation/DejaVu Sans for visual consistency
  between body text and diagram labels.
- mitsue_todo.pdf: 2-page A3 landscape (front/back of one A3 sheet) compiled
  from mitsue_todo.xlsx — Master To-Do on page 1, Legal Checklist + Risk
  Register side-by-side on page 2, with phase color bands and Japanese
  glyph support.
- mitsue_todo.xlsx: minor content update; remove unused files.zip.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mitsue_todo.xlsx
+++ b/mitsue_todo.xlsx
@@ -1,31 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="0"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Master To-Do" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Legal Checklist" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Risk Register" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Master To-Do" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legal Checklist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Risk Register" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Master To-Do'!$A$4:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master To-Do'!$A$4:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master To-Do'!$A$4:$G$60</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
   <si>
     <t xml:space="preserve">Mitsue Project — Master To-Do List</t>
   </si>
@@ -33,25 +31,25 @@
     <t xml:space="preserve">Status options: Not started • In progress • Blocked • Done</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Due</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Due</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 0</t>
@@ -66,7 +64,7 @@
     <t xml:space="preserve">Not started</t>
   </si>
   <si>
-    <t xml:space="preserve">High</t>
+    <t>High</t>
   </si>
   <si>
     <t xml:space="preserve">Listen first, present second</t>
@@ -81,13 +79,13 @@
     <t xml:space="preserve">Identify and confirm Japanese co-founder</t>
   </si>
   <si>
-    <t xml:space="preserve">Rob</t>
+    <t>Rob</t>
   </si>
   <si>
     <t xml:space="preserve">In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">Critical</t>
+    <t>Critical</t>
   </si>
   <si>
     <t xml:space="preserve">Most important single decision</t>
@@ -102,7 +100,7 @@
     <t xml:space="preserve">Quiet conversations with 2–3 sympathetic landowners</t>
   </si>
   <si>
-    <t xml:space="preserve">Medium</t>
+    <t>Medium</t>
   </si>
   <si>
     <t xml:space="preserve">Gauge sugi harvesting interest</t>
@@ -129,7 +127,7 @@
     <t xml:space="preserve">Open project Slack/Signal/email list</t>
   </si>
   <si>
-    <t xml:space="preserve">Low</t>
+    <t>Low</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 1</t>
@@ -138,13 +136,13 @@
     <t xml:space="preserve">Draft 定款 (articles of incorporation)</t>
   </si>
   <si>
-    <t xml:space="preserve">行政書士</t>
+    <t>行政書士</t>
   </si>
   <si>
     <t xml:space="preserve">Notarize 定款</t>
   </si>
   <si>
-    <t xml:space="preserve">~¥50,000</t>
+    <t>~¥50,000</t>
   </si>
   <si>
     <t xml:space="preserve">Register 一般社団法人 with Legal Affairs Bureau</t>
@@ -156,7 +154,7 @@
     <t xml:space="preserve">Tax registration (法人税, 消費税)</t>
   </si>
   <si>
-    <t xml:space="preserve">税理士</t>
+    <t>税理士</t>
   </si>
   <si>
     <t xml:space="preserve">Open corporate bank account</t>
@@ -180,7 +178,7 @@
     <t xml:space="preserve">Commission Energy Systems Feasibility Study</t>
   </si>
   <si>
-    <t xml:space="preserve">¥2–4M</t>
+    <t>¥2–4M</t>
   </si>
   <si>
     <t xml:space="preserve">Commission Building &amp; Site Assessment</t>
@@ -234,7 +232,7 @@
     <t xml:space="preserve">Landowner partnership template contract</t>
   </si>
   <si>
-    <t xml:space="preserve">弁護士</t>
+    <t>弁護士</t>
   </si>
   <si>
     <t xml:space="preserve">Vendor selection — biomass equipment</t>
@@ -342,13 +340,13 @@
     <t xml:space="preserve">Rep Dir + Rob</t>
   </si>
   <si>
-    <t xml:space="preserve">Cross-cutting</t>
+    <t>Cross-cutting</t>
   </si>
   <si>
     <t xml:space="preserve">Diversify funding — never depend on one source</t>
   </si>
   <si>
-    <t xml:space="preserve">Ongoing</t>
+    <t>Ongoing</t>
   </si>
   <si>
     <t xml:space="preserve">Risk mitigation</t>
@@ -369,13 +367,13 @@
     <t xml:space="preserve">Legal &amp; Regulatory Checklist</t>
   </si>
   <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done?</t>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Done?</t>
   </si>
   <si>
     <t xml:space="preserve">Entity &amp; Tax</t>
@@ -386,7 +384,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">一般社団法人 </t>
     </r>
@@ -395,14 +392,12 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">incorporation</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">☐</t>
+      </rPr>
+      <t>incorporation</t>
+    </r>
+  </si>
+  <si>
+    <t>☐</t>
   </si>
   <si>
     <r>
@@ -410,8 +405,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Tax registration (</t>
     </r>
@@ -420,17 +413,14 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">法人税</t>
+      </rPr>
+      <t>法人税</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -439,19 +429,16 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">消費税</t>
+      </rPr>
+      <t>消費税</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
+      </rPr>
+      <t>)</t>
     </r>
   </si>
   <si>
@@ -463,8 +450,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Accounting system (e.g. </t>
     </r>
@@ -473,23 +458,20 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">弥生会計</t>
+      </rPr>
+      <t>弥生会計</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Permits</t>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>Permits</t>
   </si>
   <si>
     <r>
@@ -497,8 +479,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Forestry permit — </t>
     </r>
@@ -507,7 +487,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">伐採届出 </t>
     </r>
@@ -516,8 +495,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">(Forest Act)</t>
     </r>
@@ -528,8 +505,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Land use coordination — </t>
     </r>
@@ -538,7 +513,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">農業委員会 </t>
     </r>
@@ -547,8 +521,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">if agricultural land</t>
     </r>
@@ -559,8 +531,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Building conversion — </t>
     </r>
@@ -569,9 +539,8 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">建築基準法</t>
+      </rPr>
+      <t>建築基準法</t>
     </r>
   </si>
   <si>
@@ -580,8 +549,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Fire &amp; safety — </t>
     </r>
@@ -590,7 +557,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">消防 </t>
     </r>
@@ -599,8 +565,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">approvals for biomass</t>
     </r>
@@ -611,8 +575,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Electrical — </t>
     </r>
@@ -621,7 +583,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">電気事業法 </t>
     </r>
@@ -630,10 +591,8 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">compliance</t>
+      </rPr>
+      <t>compliance</t>
     </r>
   </si>
   <si>
@@ -645,8 +604,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Environmental impact — </t>
     </r>
@@ -655,7 +612,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">環境アセスメント </t>
     </r>
@@ -664,8 +620,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">(if scale triggers)</t>
     </r>
@@ -682,8 +636,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Engage </t>
     </r>
@@ -692,7 +644,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">行政書士 </t>
     </r>
@@ -701,8 +652,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">(Nara-based ideal)</t>
     </r>
@@ -713,8 +662,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Engage </t>
     </r>
@@ -723,7 +670,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">公認会計士 </t>
     </r>
@@ -732,8 +678,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">/ </t>
     </r>
@@ -742,9 +686,8 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">税理士</t>
+      </rPr>
+      <t>税理士</t>
     </r>
   </si>
   <si>
@@ -753,7 +696,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
       </rPr>
       <t xml:space="preserve">弁護士 </t>
     </r>
@@ -762,8 +704,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">consult — landowner contracts</t>
     </r>
@@ -775,16 +715,16 @@
     <t xml:space="preserve">Risk Register</t>
   </si>
   <si>
-    <t xml:space="preserve">Risk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Likelihood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitigation</t>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>Likelihood</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Mitigation</t>
   </si>
   <si>
     <t xml:space="preserve">Local community resistance</t>
@@ -844,94 +784,68 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="12">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="11">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.000000"/>
       <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <b/>
+      <sz val="26.000000"/>
+      <name val="Liberation Sans"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Montserrat Thin"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <i/>
+      <sz val="11.000000"/>
+      <color rgb="FF555555"/>
+      <name val="Liberation Sans"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <name val="Montserrat Thin"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <b/>
+      <sz val="11.000000"/>
+      <color theme="0" tint="0"/>
+      <name val="Open Sans"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="11"/>
-      <color rgb="FF555555"/>
-      <name val="Montserrat Thin"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <b/>
+      <sz val="11.000000"/>
+      <color theme="1" tint="0"/>
+      <name val="Open Sans"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Montserrat Thin"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <sz val="11.000000"/>
+      <color theme="1" tint="0"/>
+      <name val="Open Sans"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Montserrat Thin"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <b/>
+      <sz val="14.000000"/>
+      <name val="Cambria"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="14"/>
+      <b/>
+      <sz val="11.000000"/>
+      <color indexed="65"/>
       <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -940,20 +854,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2C7A8C"/>
-        <bgColor rgb="FF008080"/>
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor theme="0" tint="-0.34998626667073579"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F4F8"/>
-        <bgColor rgb="FFEAEDED"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD6EAF8"/>
-        <bgColor rgb="FFEAEDED"/>
+        <fgColor theme="0" tint="0"/>
+        <bgColor theme="0" tint="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2C7A8C"/>
+        <bgColor indexed="21"/>
       </patternFill>
     </fill>
     <fill>
@@ -964,8 +884,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5CBA7"/>
-        <bgColor rgb="FFFADBD8"/>
+        <fgColor rgb="FFFADBD8"/>
+        <bgColor rgb="FFEBDEF0"/>
       </patternFill>
     </fill>
     <fill>
@@ -974,28 +894,16 @@
         <bgColor rgb="FFF5CBA7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEBDEF0"/>
-        <bgColor rgb="FFEAEDED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFADBD8"/>
-        <bgColor rgb="FFEBDEF0"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FF888888"/>
       </left>
@@ -1008,364 +916,134 @@
       <bottom style="thin">
         <color rgb="FF888888"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="6">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellXfs count="16">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="5" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="6" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="7" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="7" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="8" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="9" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="10" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF2C7A8C"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6EAF8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE8F4F8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEBDEF0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF5CBA7"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCEB6C"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCF3CF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEAEDED"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCEB6C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCF3CF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFADBD8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEAEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF2C7A8C"/>
-      <rgbColor rgb="FFFADBD8"/>
-      <rgbColor rgb="FF888888"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFCF3CF"/>
-      <rgbColor rgb="FFD6EAF8"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFEBDEF0"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFE8F4F8"/>
-      <rgbColor rgb="FFEAEDED"/>
-      <rgbColor rgb="FFFCEB6C"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF5CBA7"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF555555"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1373,17 +1051,300 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1407,7 +1368,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1428,7 +1388,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1476,10 +1435,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:path path="circle"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1494,36 +1450,34 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:path path="circle"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="50"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="1" width="8.68"/>
+    <col customWidth="1" min="1" max="1" style="1" width="14"/>
+    <col customWidth="1" min="2" max="2" style="1" width="77.28125"/>
+    <col customWidth="1" min="3" max="3" style="1" width="22"/>
+    <col customWidth="1" min="4" max="4" style="1" width="21.8515625"/>
+    <col customWidth="1" min="5" max="5" style="1" width="12"/>
+    <col customWidth="1" min="6" max="6" style="1" width="11"/>
+    <col customWidth="1" min="7" max="7" style="1" width="50"/>
+    <col customWidth="0" min="8" max="16384" style="1" width="8.6799999999999997"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="30.75">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1534,7 +1488,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="15">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1545,7 +1499,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
@@ -1568,7 +1522,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" ht="16.5">
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
@@ -1589,8 +1543,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
+    <row r="6" ht="16.5">
+      <c r="A6" s="7"/>
       <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
@@ -1606,8 +1560,8 @@
       </c>
       <c r="G6" s="6"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
+    <row r="7" ht="16.5">
+      <c r="A7" s="7"/>
       <c r="B7" s="6" t="s">
         <v>17</v>
       </c>
@@ -1625,8 +1579,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
+    <row r="8" ht="16.5">
+      <c r="A8" s="7"/>
       <c r="B8" s="6" t="s">
         <v>22</v>
       </c>
@@ -1644,8 +1598,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
+    <row r="9" ht="16.5">
+      <c r="A9" s="7"/>
       <c r="B9" s="6" t="s">
         <v>24</v>
       </c>
@@ -1663,8 +1617,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
+    <row r="10" ht="16.5">
+      <c r="A10" s="7"/>
       <c r="B10" s="6" t="s">
         <v>27</v>
       </c>
@@ -1680,8 +1634,8 @@
       </c>
       <c r="G10" s="6"/>
     </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
+    <row r="11" ht="16.5">
+      <c r="A11" s="7"/>
       <c r="B11" s="6" t="s">
         <v>28</v>
       </c>
@@ -1699,8 +1653,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
+    <row r="12" ht="16.5">
+      <c r="A12" s="7"/>
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
@@ -1716,8 +1670,8 @@
       </c>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
+    <row r="13" ht="16.5">
+      <c r="A13" s="7"/>
       <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
@@ -1735,8 +1689,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
+    <row r="14" ht="16.5">
+      <c r="A14" s="7"/>
       <c r="B14" s="6" t="s">
         <v>33</v>
       </c>
@@ -1752,8 +1706,8 @@
       </c>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="15" ht="16.5">
+      <c r="A15" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -1771,8 +1725,8 @@
       </c>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
+    <row r="16" ht="16.5">
+      <c r="A16" s="7"/>
       <c r="B16" s="6" t="s">
         <v>38</v>
       </c>
@@ -1790,8 +1744,8 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
+    <row r="17" ht="16.5">
+      <c r="A17" s="7"/>
       <c r="B17" s="6" t="s">
         <v>40</v>
       </c>
@@ -1809,8 +1763,8 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
+    <row r="18" ht="16.5">
+      <c r="A18" s="7"/>
       <c r="B18" s="6" t="s">
         <v>42</v>
       </c>
@@ -1826,8 +1780,8 @@
       </c>
       <c r="G18" s="6"/>
     </row>
-    <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8"/>
+    <row r="19" ht="33">
+      <c r="A19" s="7"/>
       <c r="B19" s="6" t="s">
         <v>44</v>
       </c>
@@ -1843,8 +1797,8 @@
       </c>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8"/>
+    <row r="20" ht="16.5">
+      <c r="A20" s="7"/>
       <c r="B20" s="6" t="s">
         <v>46</v>
       </c>
@@ -1860,8 +1814,8 @@
       </c>
       <c r="G20" s="6"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8"/>
+    <row r="21" ht="16.5">
+      <c r="A21" s="7"/>
       <c r="B21" s="6" t="s">
         <v>47</v>
       </c>
@@ -1879,8 +1833,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8"/>
+    <row r="22" ht="16.5">
+      <c r="A22" s="7"/>
       <c r="B22" s="6" t="s">
         <v>50</v>
       </c>
@@ -1898,8 +1852,8 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8"/>
+    <row r="23" ht="16.5">
+      <c r="A23" s="7"/>
       <c r="B23" s="6" t="s">
         <v>52</v>
       </c>
@@ -1917,8 +1871,8 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8"/>
+    <row r="24" ht="16.5">
+      <c r="A24" s="7"/>
       <c r="B24" s="6" t="s">
         <v>54</v>
       </c>
@@ -1936,8 +1890,8 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8"/>
+    <row r="25" ht="33">
+      <c r="A25" s="7"/>
       <c r="B25" s="6" t="s">
         <v>56</v>
       </c>
@@ -1953,8 +1907,8 @@
       </c>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8"/>
+    <row r="26" ht="16.5">
+      <c r="A26" s="7"/>
       <c r="B26" s="6" t="s">
         <v>57</v>
       </c>
@@ -1970,8 +1924,8 @@
       </c>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8"/>
+    <row r="27" ht="16.5">
+      <c r="A27" s="7"/>
       <c r="B27" s="6" t="s">
         <v>58</v>
       </c>
@@ -1987,8 +1941,8 @@
       </c>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+    <row r="28" ht="33">
+      <c r="A28" s="5" t="s">
         <v>59</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -2006,8 +1960,8 @@
       </c>
       <c r="G28" s="6"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10"/>
+    <row r="29" ht="16.5">
+      <c r="A29" s="7"/>
       <c r="B29" s="6" t="s">
         <v>62</v>
       </c>
@@ -2025,8 +1979,8 @@
         <v>63</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10"/>
+    <row r="30" ht="16.5">
+      <c r="A30" s="7"/>
       <c r="B30" s="6" t="s">
         <v>64</v>
       </c>
@@ -2042,8 +1996,8 @@
       </c>
       <c r="G30" s="6"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10"/>
+    <row r="31" ht="16.5">
+      <c r="A31" s="7"/>
       <c r="B31" s="6" t="s">
         <v>65</v>
       </c>
@@ -2059,8 +2013,8 @@
       </c>
       <c r="G31" s="6"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10"/>
+    <row r="32" ht="16.5">
+      <c r="A32" s="7"/>
       <c r="B32" s="6" t="s">
         <v>66</v>
       </c>
@@ -2076,8 +2030,8 @@
       </c>
       <c r="G32" s="6"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10"/>
+    <row r="33" ht="16.5">
+      <c r="A33" s="7"/>
       <c r="B33" s="6" t="s">
         <v>67</v>
       </c>
@@ -2093,8 +2047,8 @@
       </c>
       <c r="G33" s="6"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10"/>
+    <row r="34" ht="16.5">
+      <c r="A34" s="7"/>
       <c r="B34" s="6" t="s">
         <v>68</v>
       </c>
@@ -2110,8 +2064,8 @@
       </c>
       <c r="G34" s="6"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10"/>
+    <row r="35" ht="16.5">
+      <c r="A35" s="7"/>
       <c r="B35" s="6" t="s">
         <v>70</v>
       </c>
@@ -2127,8 +2081,8 @@
       </c>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10"/>
+    <row r="36" ht="16.5">
+      <c r="A36" s="7"/>
       <c r="B36" s="6" t="s">
         <v>71</v>
       </c>
@@ -2144,8 +2098,8 @@
       </c>
       <c r="G36" s="6"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10"/>
+    <row r="37" ht="16.5">
+      <c r="A37" s="7"/>
       <c r="B37" s="6" t="s">
         <v>72</v>
       </c>
@@ -2163,8 +2117,8 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10"/>
+    <row r="38" ht="16.5">
+      <c r="A38" s="7"/>
       <c r="B38" s="6" t="s">
         <v>75</v>
       </c>
@@ -2180,8 +2134,8 @@
       </c>
       <c r="G38" s="6"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10"/>
+    <row r="39" ht="16.5">
+      <c r="A39" s="7"/>
       <c r="B39" s="6" t="s">
         <v>76</v>
       </c>
@@ -2197,8 +2151,8 @@
       </c>
       <c r="G39" s="6"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10"/>
+    <row r="40" ht="16.5">
+      <c r="A40" s="7"/>
       <c r="B40" s="6" t="s">
         <v>77</v>
       </c>
@@ -2214,8 +2168,8 @@
       </c>
       <c r="G40" s="6"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10"/>
+    <row r="41" ht="16.5">
+      <c r="A41" s="7"/>
       <c r="B41" s="6" t="s">
         <v>78</v>
       </c>
@@ -2231,8 +2185,8 @@
       </c>
       <c r="G41" s="6"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10"/>
+    <row r="42" ht="16.5">
+      <c r="A42" s="7"/>
       <c r="B42" s="6" t="s">
         <v>79</v>
       </c>
@@ -2248,8 +2202,8 @@
       </c>
       <c r="G42" s="6"/>
     </row>
-    <row r="43" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10"/>
+    <row r="43" ht="16.5">
+      <c r="A43" s="7"/>
       <c r="B43" s="6" t="s">
         <v>80</v>
       </c>
@@ -2267,8 +2221,8 @@
         <v>81</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10"/>
+    <row r="44" ht="16.5">
+      <c r="A44" s="7"/>
       <c r="B44" s="6" t="s">
         <v>82</v>
       </c>
@@ -2284,8 +2238,8 @@
       </c>
       <c r="G44" s="6"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="10"/>
+    <row r="45" ht="16.5">
+      <c r="A45" s="7"/>
       <c r="B45" s="6" t="s">
         <v>83</v>
       </c>
@@ -2301,8 +2255,8 @@
       </c>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11" t="s">
+    <row r="46" ht="16.5">
+      <c r="A46" s="5" t="s">
         <v>85</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -2320,8 +2274,8 @@
       </c>
       <c r="G46" s="6"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="12"/>
+    <row r="47" ht="16.5">
+      <c r="A47" s="7"/>
       <c r="B47" s="6" t="s">
         <v>88</v>
       </c>
@@ -2337,8 +2291,8 @@
       </c>
       <c r="G47" s="6"/>
     </row>
-    <row r="48" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="12"/>
+    <row r="48" ht="33">
+      <c r="A48" s="7"/>
       <c r="B48" s="6" t="s">
         <v>89</v>
       </c>
@@ -2356,8 +2310,8 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12"/>
+    <row r="49" ht="16.5">
+      <c r="A49" s="7"/>
       <c r="B49" s="6" t="s">
         <v>91</v>
       </c>
@@ -2373,8 +2327,8 @@
       </c>
       <c r="G49" s="6"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="12"/>
+    <row r="50" ht="16.5">
+      <c r="A50" s="7"/>
       <c r="B50" s="6" t="s">
         <v>92</v>
       </c>
@@ -2390,8 +2344,8 @@
       </c>
       <c r="G50" s="6"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12"/>
+    <row r="51" ht="16.5">
+      <c r="A51" s="7"/>
       <c r="B51" s="6" t="s">
         <v>93</v>
       </c>
@@ -2409,8 +2363,8 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="12"/>
+    <row r="52" ht="16.5">
+      <c r="A52" s="7"/>
       <c r="B52" s="6" t="s">
         <v>95</v>
       </c>
@@ -2428,8 +2382,8 @@
         <v>96</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="13" t="s">
+    <row r="53" ht="33">
+      <c r="A53" s="5" t="s">
         <v>97</v>
       </c>
       <c r="B53" s="6" t="s">
@@ -2449,8 +2403,8 @@
         <v>99</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="14"/>
+    <row r="54" ht="16.5">
+      <c r="A54" s="7"/>
       <c r="B54" s="6" t="s">
         <v>100</v>
       </c>
@@ -2466,8 +2420,8 @@
       </c>
       <c r="G54" s="6"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="14"/>
+    <row r="55" ht="16.5">
+      <c r="A55" s="7"/>
       <c r="B55" s="6" t="s">
         <v>101</v>
       </c>
@@ -2485,8 +2439,8 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="14"/>
+    <row r="56" ht="16.5">
+      <c r="A56" s="7"/>
       <c r="B56" s="6" t="s">
         <v>103</v>
       </c>
@@ -2502,8 +2456,8 @@
       </c>
       <c r="G56" s="6"/>
     </row>
-    <row r="57" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="15" t="s">
+    <row r="57" ht="33">
+      <c r="A57" s="5" t="s">
         <v>105</v>
       </c>
       <c r="B57" s="6" t="s">
@@ -2523,8 +2477,8 @@
         <v>108</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="16"/>
+    <row r="58" ht="16.5">
+      <c r="A58" s="7"/>
       <c r="B58" s="6" t="s">
         <v>109</v>
       </c>
@@ -2540,8 +2494,8 @@
       </c>
       <c r="G58" s="6"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="16"/>
+    <row r="59" ht="16.5">
+      <c r="A59" s="7"/>
       <c r="B59" s="6" t="s">
         <v>111</v>
       </c>
@@ -2557,8 +2511,8 @@
       </c>
       <c r="G59" s="6"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="16"/>
+    <row r="60" ht="16.5">
+      <c r="A60" s="7"/>
       <c r="B60" s="6" t="s">
         <v>112</v>
       </c>
@@ -2580,459 +2534,500 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:D60">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
-      <formula>$D5="Done"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
-      <formula>$D5="In progress"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
-      <formula>$D5="Blocked"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
-      <formula>$D5="Not started"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="2" aboveAverage="0" rank="0" text="" id="{00890013-00FA-48C7-B4C2-00CF0091007A}">
+            <xm:f>$D5="Done"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFCEB6C"/>
+                  <bgColor rgb="FFFCEB6C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D5:D60</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="3" aboveAverage="0" rank="0" text="" id="{003A00E6-0004-4703-9831-00EF00520031}">
+            <xm:f>$D5="In progress"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFCF3CF"/>
+                  <bgColor rgb="FFFCF3CF"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D5:D60</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="4" aboveAverage="0" rank="0" text="" id="{00230039-0030-4CDE-95FA-007F001F0078}">
+            <xm:f>$D5="Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFADBD8"/>
+                  <bgColor rgb="FFFADBD8"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D5:D60</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="5" aboveAverage="0" rank="0" text="" id="{00F3006B-004B-4079-B448-00B100D9000B}">
+            <xm:f>$D5="Not started"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFEAEDED"/>
+                  <bgColor rgb="FFEAEDED"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D5:D60</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col customWidth="1" min="1" max="1" style="0" width="16"/>
+    <col customWidth="1" min="2" max="2" style="0" width="55"/>
+    <col customWidth="1" min="3" max="3" style="0" width="8"/>
+    <col customWidth="1" min="4" max="4" style="0" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+    <row r="1" ht="17.350000000000001">
+      <c r="A1" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+    </row>
+    <row r="3" ht="15">
+      <c r="A3" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+    <row r="4" ht="17.149999999999999">
+      <c r="A4" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="19"/>
-    </row>
-    <row r="5" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="D4" s="10"/>
+    </row>
+    <row r="5" ht="17.149999999999999">
+      <c r="A5" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="19"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="D5" s="10"/>
+    </row>
+    <row r="6" ht="15">
+      <c r="A6" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="19"/>
-    </row>
-    <row r="7" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="D6" s="10"/>
+    </row>
+    <row r="7" ht="17.149999999999999">
+      <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D7" s="19"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" ht="15">
+      <c r="A8" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D8" s="19"/>
-    </row>
-    <row r="9" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" ht="17.149999999999999">
+      <c r="A9" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="19"/>
-    </row>
-    <row r="10" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="D9" s="10"/>
+    </row>
+    <row r="10" ht="17.149999999999999">
+      <c r="A10" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="19"/>
-    </row>
-    <row r="11" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="D10" s="10"/>
+    </row>
+    <row r="11" ht="17.149999999999999">
+      <c r="A11" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="19"/>
-    </row>
-    <row r="12" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" ht="17.149999999999999">
+      <c r="A12" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D12" s="19"/>
-    </row>
-    <row r="13" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" ht="17.149999999999999">
+      <c r="A13" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="19"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="D13" s="10"/>
+    </row>
+    <row r="14" ht="15">
+      <c r="A14" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D14" s="19"/>
-    </row>
-    <row r="15" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" ht="17.149999999999999">
+      <c r="A15" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="19"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" ht="15">
+      <c r="A16" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="19"/>
-    </row>
-    <row r="17" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" ht="17.149999999999999">
+      <c r="A17" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="19"/>
-    </row>
-    <row r="18" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" ht="17.149999999999999">
+      <c r="A18" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D18" s="19"/>
-    </row>
-    <row r="19" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" ht="17.149999999999999">
+      <c r="A19" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D19" s="19"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
+      <c r="D19" s="10"/>
+    </row>
+    <row r="20" ht="15">
+      <c r="A20" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D20" s="19"/>
+      <c r="D20" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col customWidth="1" min="1" max="1" style="0" width="40"/>
+    <col customWidth="1" min="2" max="2" style="0" width="12"/>
+    <col customWidth="1" min="3" max="3" style="0" width="10"/>
+    <col customWidth="1" min="4" max="4" style="0" width="55"/>
+    <col customWidth="1" min="5" max="5" style="0" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+    <row r="1" ht="17.350000000000001">
+      <c r="A1" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+    </row>
+    <row r="3" ht="15">
+      <c r="A3" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+    <row r="4" ht="15">
+      <c r="A4" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="19" t="s">
+      <c r="C4" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+    <row r="5" ht="15">
+      <c r="A5" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="B5" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="10" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+    <row r="6" ht="23.850000000000001">
+      <c r="A6" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="19" t="s">
+      <c r="C6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+    <row r="7" ht="15">
+      <c r="A7" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="19" t="s">
+      <c r="C7" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+    <row r="8" ht="15">
+      <c r="A8" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="C8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="10" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+    <row r="9" ht="15">
+      <c r="A9" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="10" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+    <row r="10" ht="17.149999999999999">
+      <c r="A10" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="22" t="s">
+      <c r="B10" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+    <row r="11" ht="15">
+      <c r="A11" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="19" t="s">
+      <c r="C11" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="10" t="s">
         <v>110</v>
       </c>
     </row>
@@ -3040,12 +3035,9 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add bilingual Q&A briefing and early-benefits framing
- New mitsue_qa_briefing (md/docx/pdf) addresses six common
  consultation questions: biomass scale and feedstock sufficiency,
  heat utilization, the data center's role as anchor offtaker,
  benefits visible before 25 years, biomass-solar complementarity,
  and cost mitigation. Bilingual (EN/JP).
- Adds an early-benefits-within-five-years table to both English
  and Japanese village onepagers, in response to feedback that the
  25-year horizon framing alone makes village-level support harder
  to gain.
- Adds a thermal-first clarification note to README §4.2 to prevent
  the common "biomass power generation" framing assumption — the
  pilot starts with a heat-recovery boiler, not electrical generation.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mitsue_todo.xlsx
+++ b/mitsue_todo.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
   <si>
     <t xml:space="preserve">Mitsue Project — Master To-Do List</t>
   </si>
@@ -112,7 +112,10 @@
     <t xml:space="preserve">Confirm advisory commitments (Joi Ito, Ray Ozzie) in writing</t>
   </si>
   <si>
-    <t xml:space="preserve">Even informal email</t>
+    <t>Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-05 confirmed in Slack private channel.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm support letter intent — Sandra Pellegrom / Dutch Consulate</t>
@@ -806,6 +809,7 @@
       <name val="Liberation Sans"/>
     </font>
     <font>
+      <b/>
       <i/>
       <sz val="11.000000"/>
       <color rgb="FF555555"/>
@@ -845,7 +849,7 @@
       <name val="Noto Sans CJK SC"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -868,6 +872,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="0"/>
         <bgColor theme="0" tint="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FF00B050"/>
       </patternFill>
     </fill>
     <fill>
@@ -929,7 +939,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -958,10 +968,14 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="7" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
     <xf fontId="8" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="9" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf fontId="9" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
@@ -977,15 +991,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
@@ -1642,21 +1656,21 @@
       <c r="C11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>12</v>
+      <c r="D11" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" ht="16.5">
       <c r="A12" s="7"/>
       <c r="B12" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>18</v>
@@ -1673,7 +1687,7 @@
     <row r="13" ht="16.5">
       <c r="A13" s="7"/>
       <c r="B13" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>18</v>
@@ -1686,13 +1700,13 @@
         <v>25</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" ht="16.5">
       <c r="A14" s="7"/>
       <c r="B14" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>18</v>
@@ -1702,19 +1716,19 @@
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G14" s="6"/>
     </row>
     <row r="15" ht="16.5">
       <c r="A15" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>12</v>
@@ -1728,10 +1742,10 @@
     <row r="16" ht="16.5">
       <c r="A16" s="7"/>
       <c r="B16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>12</v>
@@ -1741,16 +1755,16 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" ht="16.5">
       <c r="A17" s="7"/>
       <c r="B17" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>12</v>
@@ -1760,16 +1774,16 @@
         <v>20</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" ht="16.5">
       <c r="A18" s="7"/>
       <c r="B18" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>12</v>
@@ -1783,10 +1797,10 @@
     <row r="19" ht="33">
       <c r="A19" s="7"/>
       <c r="B19" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>12</v>
@@ -1800,10 +1814,10 @@
     <row r="20" ht="16.5">
       <c r="A20" s="7"/>
       <c r="B20" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>12</v>
@@ -1817,10 +1831,10 @@
     <row r="21" ht="16.5">
       <c r="A21" s="7"/>
       <c r="B21" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>12</v>
@@ -1830,16 +1844,16 @@
         <v>20</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" ht="16.5">
       <c r="A22" s="7"/>
       <c r="B22" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>12</v>
@@ -1849,16 +1863,16 @@
         <v>20</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" ht="16.5">
       <c r="A23" s="7"/>
       <c r="B23" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>12</v>
@@ -1868,16 +1882,16 @@
         <v>20</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" ht="16.5">
       <c r="A24" s="7"/>
       <c r="B24" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>12</v>
@@ -1887,16 +1901,16 @@
         <v>13</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" ht="33">
       <c r="A25" s="7"/>
       <c r="B25" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>12</v>
@@ -1910,7 +1924,7 @@
     <row r="26" ht="16.5">
       <c r="A26" s="7"/>
       <c r="B26" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>18</v>
@@ -1927,7 +1941,7 @@
     <row r="27" ht="16.5">
       <c r="A27" s="7"/>
       <c r="B27" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>18</v>
@@ -1943,13 +1957,13 @@
     </row>
     <row r="28" ht="33">
       <c r="A28" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>12</v>
@@ -1963,10 +1977,10 @@
     <row r="29" ht="16.5">
       <c r="A29" s="7"/>
       <c r="B29" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>12</v>
@@ -1976,16 +1990,16 @@
         <v>13</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" ht="16.5">
       <c r="A30" s="7"/>
       <c r="B30" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>12</v>
@@ -1999,10 +2013,10 @@
     <row r="31" ht="16.5">
       <c r="A31" s="7"/>
       <c r="B31" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>12</v>
@@ -2016,10 +2030,10 @@
     <row r="32" ht="16.5">
       <c r="A32" s="7"/>
       <c r="B32" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>12</v>
@@ -2033,10 +2047,10 @@
     <row r="33" ht="16.5">
       <c r="A33" s="7"/>
       <c r="B33" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>12</v>
@@ -2050,10 +2064,10 @@
     <row r="34" ht="16.5">
       <c r="A34" s="7"/>
       <c r="B34" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>12</v>
@@ -2067,10 +2081,10 @@
     <row r="35" ht="16.5">
       <c r="A35" s="7"/>
       <c r="B35" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>12</v>
@@ -2084,10 +2098,10 @@
     <row r="36" ht="16.5">
       <c r="A36" s="7"/>
       <c r="B36" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>12</v>
@@ -2101,10 +2115,10 @@
     <row r="37" ht="16.5">
       <c r="A37" s="7"/>
       <c r="B37" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>12</v>
@@ -2114,16 +2128,16 @@
         <v>20</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" ht="16.5">
       <c r="A38" s="7"/>
       <c r="B38" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>12</v>
@@ -2137,10 +2151,10 @@
     <row r="39" ht="16.5">
       <c r="A39" s="7"/>
       <c r="B39" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>12</v>
@@ -2154,10 +2168,10 @@
     <row r="40" ht="16.5">
       <c r="A40" s="7"/>
       <c r="B40" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>12</v>
@@ -2171,7 +2185,7 @@
     <row r="41" ht="16.5">
       <c r="A41" s="7"/>
       <c r="B41" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>18</v>
@@ -2188,7 +2202,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="7"/>
       <c r="B42" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>18</v>
@@ -2205,7 +2219,7 @@
     <row r="43" ht="16.5">
       <c r="A43" s="7"/>
       <c r="B43" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>18</v>
@@ -2218,13 +2232,13 @@
         <v>25</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" ht="16.5">
       <c r="A44" s="7"/>
       <c r="B44" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>16</v>
@@ -2241,10 +2255,10 @@
     <row r="45" ht="16.5">
       <c r="A45" s="7"/>
       <c r="B45" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>12</v>
@@ -2257,13 +2271,13 @@
     </row>
     <row r="46" ht="16.5">
       <c r="A46" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>12</v>
@@ -2277,10 +2291,10 @@
     <row r="47" ht="16.5">
       <c r="A47" s="7"/>
       <c r="B47" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>12</v>
@@ -2294,10 +2308,10 @@
     <row r="48" ht="33">
       <c r="A48" s="7"/>
       <c r="B48" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>12</v>
@@ -2307,16 +2321,16 @@
         <v>20</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" ht="16.5">
       <c r="A49" s="7"/>
       <c r="B49" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>12</v>
@@ -2330,10 +2344,10 @@
     <row r="50" ht="16.5">
       <c r="A50" s="7"/>
       <c r="B50" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>12</v>
@@ -2347,10 +2361,10 @@
     <row r="51" ht="16.5">
       <c r="A51" s="7"/>
       <c r="B51" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>12</v>
@@ -2360,16 +2374,16 @@
         <v>25</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" ht="16.5">
       <c r="A52" s="7"/>
       <c r="B52" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>12</v>
@@ -2379,18 +2393,18 @@
         <v>25</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" ht="33">
       <c r="A53" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>12</v>
@@ -2400,16 +2414,16 @@
         <v>13</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54" ht="16.5">
       <c r="A54" s="7"/>
       <c r="B54" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>12</v>
@@ -2423,7 +2437,7 @@
     <row r="55" ht="16.5">
       <c r="A55" s="7"/>
       <c r="B55" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>18</v>
@@ -2436,16 +2450,16 @@
         <v>25</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" ht="16.5">
       <c r="A56" s="7"/>
       <c r="B56" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>12</v>
@@ -2458,32 +2472,32 @@
     </row>
     <row r="57" ht="33">
       <c r="A57" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E57" s="6"/>
       <c r="F57" s="6" t="s">
         <v>20</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="58" ht="16.5">
       <c r="A58" s="7"/>
       <c r="B58" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>12</v>
@@ -2497,13 +2511,13 @@
     <row r="59" ht="16.5">
       <c r="A59" s="7"/>
       <c r="B59" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C59" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C59" s="6" t="s">
-        <v>110</v>
-      </c>
       <c r="D59" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E59" s="6"/>
       <c r="F59" s="6" t="s">
@@ -2514,13 +2528,13 @@
     <row r="60" ht="16.5">
       <c r="A60" s="7"/>
       <c r="B60" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E60" s="6"/>
       <c r="F60" s="6" t="s">
@@ -2542,7 +2556,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="2" aboveAverage="0" rank="0" text="" id="{00890013-00FA-48C7-B4C2-00CF0091007A}">
+          <x14:cfRule type="expression" priority="2" aboveAverage="0" rank="0" text="" id="{00CF007C-0079-458C-905A-000B0083003F}">
             <xm:f>$D5="Done"</xm:f>
             <x14:dxf>
               <fill>
@@ -2556,7 +2570,7 @@
           <xm:sqref>D5:D60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="3" aboveAverage="0" rank="0" text="" id="{003A00E6-0004-4703-9831-00EF00520031}">
+          <x14:cfRule type="expression" priority="3" aboveAverage="0" rank="0" text="" id="{00F40040-0005-4BC1-A3B1-004400970075}">
             <xm:f>$D5="In progress"</xm:f>
             <x14:dxf>
               <fill>
@@ -2570,7 +2584,7 @@
           <xm:sqref>D5:D60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="4" aboveAverage="0" rank="0" text="" id="{00230039-0030-4CDE-95FA-007F001F0078}">
+          <x14:cfRule type="expression" priority="4" aboveAverage="0" rank="0" text="" id="{00D6009D-00F8-49C0-A38D-00E300BC0089}">
             <xm:f>$D5="Blocked"</xm:f>
             <x14:dxf>
               <fill>
@@ -2584,7 +2598,7 @@
           <xm:sqref>D5:D60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="5" aboveAverage="0" rank="0" text="" id="{00F3006B-004B-4079-B448-00B100D9000B}">
+          <x14:cfRule type="expression" priority="5" aboveAverage="0" rank="0" text="" id="{00AB00C1-000B-4F6C-950B-0066005F0003}">
             <xm:f>$D5="Not started"</xm:f>
             <x14:dxf>
               <fill>
@@ -2596,6 +2610,62 @@
             </x14:dxf>
           </x14:cfRule>
           <xm:sqref>D5:D60</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="2" aboveAverage="0" rank="0" text="" id="{00BB00E9-00ED-4646-A810-007100CC008E}">
+            <xm:f>$D5="Done"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFCEB6C"/>
+                  <bgColor rgb="FFFCEB6C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D11</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="3" aboveAverage="0" rank="0" text="" id="{00BC003A-00DB-4333-895E-009B002D0084}">
+            <xm:f>$D5="In progress"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFCF3CF"/>
+                  <bgColor rgb="FFFCF3CF"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D11</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="4" aboveAverage="0" rank="0" text="" id="{0019002D-00FA-4E16-AEBA-005C001D0097}">
+            <xm:f>$D5="Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFADBD8"/>
+                  <bgColor rgb="FFFADBD8"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D11</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="5" aboveAverage="0" rank="0" text="" id="{002E0070-008D-459F-BCE9-00CC00940059}">
+            <xm:f>$D5="Not started"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFEAEDED"/>
+                  <bgColor rgb="FFEAEDED"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>D11</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -2618,230 +2688,230 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.350000000000001">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+    </row>
+    <row r="3" ht="15">
+      <c r="A3" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" ht="17.149999999999999">
+      <c r="A4" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" ht="17.149999999999999">
+      <c r="A5" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" ht="15">
+      <c r="A6" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" ht="17.149999999999999">
+      <c r="A7" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" s="11"/>
+    </row>
+    <row r="8" ht="15">
+      <c r="A8" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-    </row>
-    <row r="3" ht="15">
-      <c r="A3" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" ht="17.149999999999999">
-      <c r="A4" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D4" s="10"/>
-    </row>
-    <row r="5" ht="17.149999999999999">
-      <c r="A5" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B5" s="10" t="s">
+      <c r="C8" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D5" s="10"/>
-    </row>
-    <row r="6" ht="15">
-      <c r="A6" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D6" s="10"/>
-    </row>
-    <row r="7" ht="17.149999999999999">
-      <c r="A7" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D7" s="10"/>
-    </row>
-    <row r="8" ht="15">
-      <c r="A8" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D8" s="10"/>
+      <c r="D8" s="11"/>
     </row>
     <row r="9" ht="17.149999999999999">
-      <c r="A9" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B9" s="10" t="s">
+      <c r="A9" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D9" s="10"/>
+      <c r="B9" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="11"/>
     </row>
     <row r="10" ht="17.149999999999999">
-      <c r="A10" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D10" s="10"/>
+      <c r="A10" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="11"/>
     </row>
     <row r="11" ht="17.149999999999999">
-      <c r="A11" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D11" s="10"/>
+      <c r="A11" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="11"/>
     </row>
     <row r="12" ht="17.149999999999999">
-      <c r="A12" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D12" s="10"/>
+      <c r="A12" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" ht="17.149999999999999">
-      <c r="A13" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D13" s="10"/>
+      <c r="A13" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" ht="15">
-      <c r="A14" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D14" s="10"/>
+      <c r="A14" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" ht="17.149999999999999">
-      <c r="A15" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D15" s="10"/>
+      <c r="A15" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="11"/>
     </row>
     <row r="16" ht="15">
-      <c r="A16" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D16" s="10"/>
+      <c r="A16" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" ht="17.149999999999999">
-      <c r="A17" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="A17" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D17" s="10"/>
+      <c r="B17" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" ht="17.149999999999999">
-      <c r="A18" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D18" s="10"/>
+      <c r="A18" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" ht="17.149999999999999">
-      <c r="A19" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D19" s="10"/>
+      <c r="A19" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" ht="15">
-      <c r="A20" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="D20" s="10"/>
+      <c r="A20" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2870,165 +2940,165 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.350000000000001">
-      <c r="A1" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="A1" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="3" ht="15">
-      <c r="A3" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" ht="15">
-      <c r="A4" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B4" s="13" t="s">
+      <c r="A4" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>110</v>
+      <c r="C4" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="A5" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="B5" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>146</v>
       </c>
+      <c r="E5" s="11" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="6" ht="23.850000000000001">
-      <c r="A6" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B6" s="13" t="s">
+      <c r="A6" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="C6" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="A7" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="B7" s="13" t="s">
+      <c r="A7" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>110</v>
+      <c r="C7" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="A8" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="B8" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>153</v>
       </c>
+      <c r="E8" s="11" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="9" ht="15">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="B9" s="13" t="s">
+    </row>
+    <row r="10" ht="17.149999999999999">
+      <c r="A10" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="D10" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" ht="15">
+      <c r="A11" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="10" ht="17.149999999999999">
-      <c r="A10" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" ht="15">
-      <c r="A11" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>110</v>
+      <c r="C11" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>